<commit_message>
Agrega RIPTE real (deflactado por el IPC nacional)
Las series derivadas pueden depender de varias bases.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WiZx484kRcrrNZ4YGQ81g
</commit_message>
<xml_diff>
--- a/data/excel/emae_letras_desest.xlsx
+++ b/data/excel/emae_letras_desest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Niveles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datos de la serie" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos de la serie" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,16 +22,13 @@
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="166" formatCode="mmm-yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -438,94 +426,94 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>A - Agricultura, ganadería, caza y silvicultura, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>A - Agricultura, ganadería, caza y silvicultura, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>C - Explotación de minas y canteras, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>C - Explotación de minas y canteras, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>D - Industria manufacturera, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>D - Industria manufacturera, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>E - Electricidad, gas y agua, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>E - Electricidad, gas y agua, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>F - Construcción, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>F - Construcción, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>G - Comercio mayorista, minorista y reparaciones, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>G - Comercio mayorista, minorista y reparaciones, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>I - Transporte y comunicaciones, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>I - Transporte y comunicaciones, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>J - Intermediación financiera, desestacionalizada (propia, X-13)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>J - Intermediación financiera, desestacionalizada (propia, X-13), var. % mensual</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>37987</v>
       </c>
       <c r="B2" t="n">
@@ -562,7 +550,7 @@
       <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38018</v>
       </c>
       <c r="B3" t="n">
@@ -615,7 +603,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38047</v>
       </c>
       <c r="B4" t="n">
@@ -668,7 +656,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38078</v>
       </c>
       <c r="B5" t="n">
@@ -721,7 +709,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38108</v>
       </c>
       <c r="B6" t="n">
@@ -774,7 +762,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38139</v>
       </c>
       <c r="B7" t="n">
@@ -827,7 +815,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38169</v>
       </c>
       <c r="B8" t="n">
@@ -880,7 +868,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38200</v>
       </c>
       <c r="B9" t="n">
@@ -933,7 +921,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38231</v>
       </c>
       <c r="B10" t="n">
@@ -986,7 +974,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38261</v>
       </c>
       <c r="B11" t="n">
@@ -1039,7 +1027,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>38292</v>
       </c>
       <c r="B12" t="n">
@@ -1092,7 +1080,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>38322</v>
       </c>
       <c r="B13" t="n">
@@ -1145,7 +1133,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>38353</v>
       </c>
       <c r="B14" t="n">
@@ -1198,7 +1186,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>38384</v>
       </c>
       <c r="B15" t="n">
@@ -1251,7 +1239,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>38412</v>
       </c>
       <c r="B16" t="n">
@@ -1304,7 +1292,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>38443</v>
       </c>
       <c r="B17" t="n">
@@ -1357,7 +1345,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>38473</v>
       </c>
       <c r="B18" t="n">
@@ -1410,7 +1398,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>38504</v>
       </c>
       <c r="B19" t="n">
@@ -1463,7 +1451,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>38534</v>
       </c>
       <c r="B20" t="n">
@@ -1516,7 +1504,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>38565</v>
       </c>
       <c r="B21" t="n">
@@ -1569,7 +1557,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>38596</v>
       </c>
       <c r="B22" t="n">
@@ -1622,7 +1610,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>38626</v>
       </c>
       <c r="B23" t="n">
@@ -1675,7 +1663,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>38657</v>
       </c>
       <c r="B24" t="n">
@@ -1728,7 +1716,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>38687</v>
       </c>
       <c r="B25" t="n">
@@ -1781,7 +1769,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B26" t="n">
@@ -1834,7 +1822,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B27" t="n">
@@ -1887,7 +1875,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B28" t="n">
@@ -1940,7 +1928,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B29" t="n">
@@ -1993,7 +1981,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B30" t="n">
@@ -2046,7 +2034,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B31" t="n">
@@ -2099,7 +2087,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B32" t="n">
@@ -2152,7 +2140,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B33" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B34" t="n">
@@ -2258,7 +2246,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B35" t="n">
@@ -2311,7 +2299,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B36" t="n">
@@ -2364,7 +2352,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B37" t="n">
@@ -2417,7 +2405,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B38" t="n">
@@ -2470,7 +2458,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B39" t="n">
@@ -2523,7 +2511,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B40" t="n">
@@ -2576,7 +2564,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B41" t="n">
@@ -2629,7 +2617,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B42" t="n">
@@ -2682,7 +2670,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B43" t="n">
@@ -2735,7 +2723,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B44" t="n">
@@ -2788,7 +2776,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B45" t="n">
@@ -2841,7 +2829,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B46" t="n">
@@ -2894,7 +2882,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B47" t="n">
@@ -2947,7 +2935,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B48" t="n">
@@ -3000,7 +2988,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B49" t="n">
@@ -3053,7 +3041,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B50" t="n">
@@ -3106,7 +3094,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B51" t="n">
@@ -3159,7 +3147,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B52" t="n">
@@ -3212,7 +3200,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B53" t="n">
@@ -3265,7 +3253,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B54" t="n">
@@ -3318,7 +3306,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B55" t="n">
@@ -3371,7 +3359,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B56" t="n">
@@ -3424,7 +3412,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B57" t="n">
@@ -3477,7 +3465,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B58" t="n">
@@ -3530,7 +3518,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B59" t="n">
@@ -3583,7 +3571,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B60" t="n">
@@ -3636,7 +3624,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B61" t="n">
@@ -3689,7 +3677,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B62" t="n">
@@ -3742,7 +3730,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B63" t="n">
@@ -3795,7 +3783,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B64" t="n">
@@ -3848,7 +3836,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B65" t="n">
@@ -3901,7 +3889,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B66" t="n">
@@ -3954,7 +3942,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B67" t="n">
@@ -4007,7 +3995,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B68" t="n">
@@ -4060,7 +4048,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B69" t="n">
@@ -4113,7 +4101,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B70" t="n">
@@ -4166,7 +4154,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B71" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B72" t="n">
@@ -4272,7 +4260,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B73" t="n">
@@ -4325,7 +4313,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B74" t="n">
@@ -4378,7 +4366,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B75" t="n">
@@ -4431,7 +4419,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B76" t="n">
@@ -4484,7 +4472,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B77" t="n">
@@ -4537,7 +4525,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B78" t="n">
@@ -4590,7 +4578,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B79" t="n">
@@ -4643,7 +4631,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B80" t="n">
@@ -4696,7 +4684,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B81" t="n">
@@ -4749,7 +4737,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B82" t="n">
@@ -4802,7 +4790,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B83" t="n">
@@ -4855,7 +4843,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B84" t="n">
@@ -4908,7 +4896,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B85" t="n">
@@ -4961,7 +4949,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B86" t="n">
@@ -5014,7 +5002,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B87" t="n">
@@ -5067,7 +5055,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B88" t="n">
@@ -5120,7 +5108,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B89" t="n">
@@ -5173,7 +5161,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B90" t="n">
@@ -5226,7 +5214,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B91" t="n">
@@ -5279,7 +5267,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B92" t="n">
@@ -5332,7 +5320,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B93" t="n">
@@ -5385,7 +5373,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B94" t="n">
@@ -5438,7 +5426,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B95" t="n">
@@ -5491,7 +5479,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B96" t="n">
@@ -5544,7 +5532,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B97" t="n">
@@ -5597,7 +5585,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B98" t="n">
@@ -5650,7 +5638,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B99" t="n">
@@ -5703,7 +5691,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B100" t="n">
@@ -5756,7 +5744,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B101" t="n">
@@ -5809,7 +5797,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B102" t="n">
@@ -5862,7 +5850,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B103" t="n">
@@ -5915,7 +5903,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B104" t="n">
@@ -5968,7 +5956,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B105" t="n">
@@ -6021,7 +6009,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B106" t="n">
@@ -6074,7 +6062,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B107" t="n">
@@ -6127,7 +6115,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B108" t="n">
@@ -6180,7 +6168,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B109" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B110" t="n">
@@ -6286,7 +6274,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B111" t="n">
@@ -6339,7 +6327,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B112" t="n">
@@ -6392,7 +6380,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B113" t="n">
@@ -6445,7 +6433,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B114" t="n">
@@ -6498,7 +6486,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B115" t="n">
@@ -6551,7 +6539,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B116" t="n">
@@ -6604,7 +6592,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B117" t="n">
@@ -6657,7 +6645,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B118" t="n">
@@ -6710,7 +6698,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B119" t="n">
@@ -6763,7 +6751,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B120" t="n">
@@ -6816,7 +6804,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B121" t="n">
@@ -6869,7 +6857,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B122" t="n">
@@ -6922,7 +6910,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B123" t="n">
@@ -6975,7 +6963,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B124" t="n">
@@ -7028,7 +7016,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B125" t="n">
@@ -7081,7 +7069,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B126" t="n">
@@ -7134,7 +7122,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B127" t="n">
@@ -7187,7 +7175,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B128" t="n">
@@ -7240,7 +7228,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B129" t="n">
@@ -7293,7 +7281,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B130" t="n">
@@ -7346,7 +7334,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B131" t="n">
@@ -7399,7 +7387,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B132" t="n">
@@ -7452,7 +7440,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B133" t="n">
@@ -7505,7 +7493,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B134" t="n">
@@ -7558,7 +7546,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B135" t="n">
@@ -7611,7 +7599,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B136" t="n">
@@ -7664,7 +7652,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B137" t="n">
@@ -7717,7 +7705,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B138" t="n">
@@ -7770,7 +7758,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B139" t="n">
@@ -7823,7 +7811,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B140" t="n">
@@ -7876,7 +7864,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B141" t="n">
@@ -7929,7 +7917,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B142" t="n">
@@ -7982,7 +7970,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B143" t="n">
@@ -8035,7 +8023,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B144" t="n">
@@ -8088,7 +8076,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B145" t="n">
@@ -8141,7 +8129,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B146" t="n">
@@ -8194,7 +8182,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B147" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B148" t="n">
@@ -8300,7 +8288,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B149" t="n">
@@ -8353,7 +8341,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B150" t="n">
@@ -8406,7 +8394,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B151" t="n">
@@ -8459,7 +8447,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B152" t="n">
@@ -8512,7 +8500,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B153" t="n">
@@ -8565,7 +8553,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B154" t="n">
@@ -8618,7 +8606,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B155" t="n">
@@ -8671,7 +8659,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B156" t="n">
@@ -8724,7 +8712,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B157" t="n">
@@ -8777,7 +8765,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B158" t="n">
@@ -8830,7 +8818,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B159" t="n">
@@ -8883,7 +8871,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B160" t="n">
@@ -8936,7 +8924,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B161" t="n">
@@ -8989,7 +8977,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B162" t="n">
@@ -9042,7 +9030,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B163" t="n">
@@ -9095,7 +9083,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B164" t="n">
@@ -9148,7 +9136,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B165" t="n">
@@ -9201,7 +9189,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B166" t="n">
@@ -9254,7 +9242,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B167" t="n">
@@ -9307,7 +9295,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B168" t="n">
@@ -9360,7 +9348,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B169" t="n">
@@ -9413,7 +9401,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B170" t="n">
@@ -9466,7 +9454,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B171" t="n">
@@ -9519,7 +9507,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B172" t="n">
@@ -9572,7 +9560,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B173" t="n">
@@ -9625,7 +9613,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B174" t="n">
@@ -9678,7 +9666,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B175" t="n">
@@ -9731,7 +9719,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B176" t="n">
@@ -9784,7 +9772,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B177" t="n">
@@ -9837,7 +9825,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B178" t="n">
@@ -9890,7 +9878,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B179" t="n">
@@ -9943,7 +9931,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B180" t="n">
@@ -9996,7 +9984,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B181" t="n">
@@ -10049,7 +10037,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B182" t="n">
@@ -10102,7 +10090,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B183" t="n">
@@ -10155,7 +10143,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B184" t="n">
@@ -10208,7 +10196,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B185" t="n">
@@ -10261,7 +10249,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B186" t="n">
@@ -10314,7 +10302,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B187" t="n">
@@ -10367,7 +10355,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B188" t="n">
@@ -10420,7 +10408,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B189" t="n">
@@ -10473,7 +10461,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B190" t="n">
@@ -10526,7 +10514,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B191" t="n">
@@ -10579,7 +10567,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B192" t="n">
@@ -10632,7 +10620,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B193" t="n">
@@ -10685,7 +10673,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B194" t="n">
@@ -10738,7 +10726,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B195" t="n">
@@ -10791,7 +10779,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B196" t="n">
@@ -10844,7 +10832,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B197" t="n">
@@ -10897,7 +10885,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B198" t="n">
@@ -10950,7 +10938,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B199" t="n">
@@ -11003,7 +10991,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B200" t="n">
@@ -11056,7 +11044,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B201" t="n">
@@ -11109,7 +11097,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B202" t="n">
@@ -11162,7 +11150,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B203" t="n">
@@ -11215,7 +11203,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B204" t="n">
@@ -11268,7 +11256,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B205" t="n">
@@ -11321,7 +11309,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B206" t="n">
@@ -11374,7 +11362,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B207" t="n">
@@ -11427,7 +11415,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B208" t="n">
@@ -11480,7 +11468,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B209" t="n">
@@ -11533,7 +11521,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B210" t="n">
@@ -11586,7 +11574,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B211" t="n">
@@ -11639,7 +11627,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B212" t="n">
@@ -11692,7 +11680,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B213" t="n">
@@ -11745,7 +11733,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B214" t="n">
@@ -11798,7 +11786,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B215" t="n">
@@ -11851,7 +11839,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B216" t="n">
@@ -11904,7 +11892,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B217" t="n">
@@ -11957,7 +11945,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B218" t="n">
@@ -12010,7 +11998,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B219" t="n">
@@ -12063,7 +12051,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B220" t="n">
@@ -12116,7 +12104,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B221" t="n">
@@ -12169,7 +12157,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B222" t="n">
@@ -12222,7 +12210,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B223" t="n">
@@ -12275,7 +12263,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B224" t="n">
@@ -12328,7 +12316,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B225" t="n">
@@ -12381,7 +12369,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B226" t="n">
@@ -12434,7 +12422,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B227" t="n">
@@ -12487,7 +12475,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B228" t="n">
@@ -12540,7 +12528,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B229" t="n">
@@ -12593,7 +12581,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B230" t="n">
@@ -12646,7 +12634,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B231" t="n">
@@ -12699,7 +12687,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B232" t="n">
@@ -12752,7 +12740,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B233" t="n">
@@ -12805,7 +12793,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B234" t="n">
@@ -12858,7 +12846,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B235" t="n">
@@ -12911,7 +12899,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B236" t="n">
@@ -12964,7 +12952,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B237" t="n">
@@ -13017,7 +13005,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B238" t="n">
@@ -13070,7 +13058,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B239" t="n">
@@ -13123,7 +13111,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B240" t="n">
@@ -13176,7 +13164,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B241" t="n">
@@ -13229,7 +13217,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B242" t="n">
@@ -13282,7 +13270,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B243" t="n">
@@ -13335,7 +13323,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B244" t="n">
@@ -13388,7 +13376,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B245" t="n">
@@ -13441,7 +13429,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B246" t="n">
@@ -13494,7 +13482,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B247" t="n">
@@ -13547,7 +13535,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n">
+      <c r="A248" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B248" t="n">
@@ -13600,7 +13588,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="2" t="n">
+      <c r="A249" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B249" t="n">
@@ -13653,7 +13641,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="n">
+      <c r="A250" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B250" t="n">
@@ -13706,7 +13694,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="2" t="n">
+      <c r="A251" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B251" t="n">
@@ -13759,7 +13747,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="n">
+      <c r="A252" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B252" t="n">
@@ -13812,7 +13800,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="n">
+      <c r="A253" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B253" t="n">
@@ -13865,7 +13853,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="n">
+      <c r="A254" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B254" t="n">
@@ -13918,7 +13906,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="n">
+      <c r="A255" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B255" t="n">
@@ -13971,7 +13959,7 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="n">
+      <c r="A256" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B256" t="n">
@@ -14024,7 +14012,7 @@
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="n">
+      <c r="A257" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B257" t="n">
@@ -14077,7 +14065,7 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="n">
+      <c r="A258" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B258" t="n">
@@ -14130,7 +14118,7 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="n">
+      <c r="A259" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B259" t="n">
@@ -14183,7 +14171,7 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="n">
+      <c r="A260" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B260" t="n">
@@ -14236,7 +14224,7 @@
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="n">
+      <c r="A261" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B261" t="n">
@@ -14289,7 +14277,7 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="n">
+      <c r="A262" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B262" t="n">
@@ -14342,7 +14330,7 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="n">
+      <c r="A263" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B263" t="n">
@@ -14395,7 +14383,7 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="n">
+      <c r="A264" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B264" t="n">
@@ -14448,7 +14436,7 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="n">
+      <c r="A265" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B265" t="n">
@@ -14501,7 +14489,7 @@
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="n">
+      <c r="A266" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B266" t="n">
@@ -14554,7 +14542,7 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="2" t="n">
+      <c r="A267" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B267" t="n">
@@ -14607,7 +14595,7 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="n">
+      <c r="A268" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B268" t="n">
@@ -14660,7 +14648,7 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n">
+      <c r="A269" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B269" t="n">
@@ -14713,7 +14701,7 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="n">
+      <c r="A270" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B270" t="n">
@@ -14766,7 +14754,7 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="n">
+      <c r="A271" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="B271" t="n">
@@ -14819,7 +14807,7 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n">
+      <c r="A272" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B272" t="n">

</xml_diff>